<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.003-01 Le bateau de papier de Mila
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.003-01.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.003-01.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>entrée puis cour après la pluie</t>
+          <t>entrée puis cour après la pluie, radiateur, manteaux, botte jaune</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mila, Sarah, maman</t>
+          <t>Mila, Sarah, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut un bateau de papier dans la flaque de la cour. Le pli est de travers. Sarah, avec ses lunettes, voit le pli. Elles soufflent sur la voile.</t>
+          <t>La laine sent la pluie. Un tic chaud. Sur le caoutchouc, un éclat de botte luit. Mila veut un bateau dans la flaque, maintenant, avec Sarah. Elle tend trop vite vers les lunettes : non. Le bateau penche, n'atteint pas. Sourire parti. Elle refuse de foncer. Merci vécu. Elle pose d'un coup : le papier reste au bord. Elle s'arrête, lit l'éclat. Un éclat de botte reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le radiateur de l'entrée fait un tic chaud. Les manteaux sentent la laine mouillée. Une botte jaune est couchée. Une goutte tombe du capuchon. Elle fait un rond sur le bois. Maman pose une feuille blanche. La feuille est un peu rêche. Tu as entendu le radiateur, Mila ? Il fait tic. Oui. Il réchauffe les manteaux. En ce moment, Mila plie la feuille. Elle veut un bateau. Il va flotter. Dans la flaque. On plie bien le milieu ? Oui. Le papier sent le bois. Un coin se replie tout seul. Mila l'aplatit avec la main. Sarah arrive près des bottes. Sarah a des lunettes neuves. Elles brillent un peu. Sarah a les cheveux courts. Son manteau est bleu vif. Venez plier toutes les deux. Tu m'aides, Sarah ? Oui. Elles plient encore. Le papier fait frrt. Un pli est trop haut. L'autre pli est trop bas. Le bateau est un peu de travers. Il penche. On peut regarder le pli. Sarah se penche. Ses lunettes aident à voir. Là. Ce pli-là. Je le vois.</t>
+          <t>La laine des manteaux sent la pluie. Ça sent mouillé, maman. Tu le sens, sur le tissu ? Oui, un peu froid. Le radiateur fait un tic chaud. Tu l'entends, près des crochets ? Oui, papa. Papa égoutte un manteau, sans parler. Une botte jaune est couchée. Sur le caoutchouc, un éclat de botte luit. Il brille, papa ! Tu le vois, sur la botte ? Oui, un petit point. Une goutte tombe du capuchon. Elle fait un rond sur le bois. Le bois est luisant. La pluie a fini, dehors. La cour brille. Il y a une flaque, Mila. Je veux un bateau, maintenant ! Un bateau de papier ? Oui, pour la flaque. Maman pose une feuille blanche. La feuille est un peu rêche. Elle sent le bois. Tu restes près des bottes ? Oui, papa. En ce moment, Mila plie la feuille trop vite. Un coin se replie tout seul. Il penche ! Le milieu, Mila ? J'y vais. Sarah arrive près des bottes. Son manteau est bleu vif. Sarah a les cheveux courts. Sarah ! Sarah a des lunettes. Elles brillent un peu. Elles brillent ! Mila avance la main vers les lunettes. Non. Sarah recule d'un pas. Oh. Mila plie toute seule, trop vite. Le papier fait frrt. Le bateau penche, de travers. Il ne tient pas. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'éclat de botte tremble, puis tient. Tu vois Sarah, Mila ? Papa s'accroupit à la même hauteur. Oui, papa. Tes mains sont froides, Mila ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le radiateur de l'entrée fait un tic chaud. Les manteaux sentent la laine mouillée. Une botte jaune est couchée. Une goutte tombe du capuchon. Elle fait un rond sur le bois. Maman pose une feuille blanche. La feuille est un peu rêche. Tu as entendu le radiateur, Mila ? Il fait tic. Oui. Il réchauffe les manteaux. En ce moment, Mila plie la feuille. Elle veut un bateau. Il va flotter. Dans la flaque. On plie bien le milieu ? Oui. Le papier sent le bois. Un coin se replie tout seul. Mila l'aplatit avec la main. Sarah arrive près des bottes. Sarah a des lunettes neuves. Elles brillent un peu. Sarah a les cheveux courts. Son manteau est bleu vif. Venez plier toutes les deux. Tu m'aides, Sarah ? Oui. Elles plient encore. Le papier fait frrt. Un pli est trop haut. L'autre pli est trop bas. Le bateau est un peu de travers. Il penche. On peut regarder le pli. Sarah se penche. Ses lunettes aident à voir. Là. Ce pli-là. Je le vois.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La laine des manteaux sent la pluie. Ça sent mouillé, maman. Tu le sens, sur le tissu ? Oui, un peu froid. Le radiateur fait un tic chaud. Tu l'entends, près des crochets ? Oui, papa. Papa égoutte un manteau, sans parler. Une botte jaune est couchée. Sur le caoutchouc, un &lt;emphasis level="moderate"&gt;éclat de botte&lt;/emphasis&gt; luit. Il brille, papa ! Tu le vois, sur la botte ? Oui, un petit point. Une goutte tombe du capuchon. Elle fait un rond sur le bois. Le bois est luisant. La pluie a fini, dehors. La cour brille. Il y a une flaque, Mila. Je veux un bateau, maintenant ! Un bateau de papier ? Oui, pour la flaque. Maman pose une feuille blanche. La feuille est un peu rêche. Elle sent le bois. Tu restes près des bottes ? Oui, papa. En ce moment, Mila plie la feuille trop vite. Un coin se replie tout seul. Il penche ! Le milieu, Mila ? J'y vais. Sarah arrive près des bottes. Son manteau est bleu vif. Sarah a les cheveux courts. Sarah ! Sarah a des lunettes. Elles brillent un peu. Elles brillent ! Mila avance la main vers les lunettes. Non. Sarah recule d'un pas. Oh. Mila plie toute seule, trop vite. Le papier fait frrt. Le bateau penche, de travers. Il ne tient pas. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'éclat de botte tremble, puis tient. Tu vois Sarah, Mila ? Papa s'accroupit à la même hauteur. Oui, papa. Tes mains sont froides, Mila ? Un peu, maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le matin, maman accompagne Inès à l'école. La cour sent les feuilles mouillées. Lila arrive. Lila a des lunettes neuves. Lila a les cheveux courts et bouclés. Lila porte un manteau bleu vif. Inès regarde. Un autre enfant laisse sortir un petit rire. Maman s'approche tout de suite. Maman dit : on ne va &lt;emphasis&gt;pas&lt;/emphasis&gt; rire de l'apparence. Les lunettes aident à voir. Les cheveux sont les cheveux. L'habit tient chaud. On joue. Inès hoche la tête. Elle va vers Lila. Inès dit : tu viens au bac à feuilles. Lila dit : oui. Elles ramassent des feuilles jaunes. Elles font un tas. La maîtresse ouvre la classe. Sur la table, il y a des perles et des fils. Inès choisit un fil rouge. Lila choisit un fil vert. Un enfant regarde encore les lunettes. Inès dit : on ne va pas rire. On enfile des perles. Lila enfile une perle ronde. Inès enfile une perle longue. Le collier de Lila brille. Le collier d'Inès brille aussi. Maman est encore près de la porte. Elle entend. Elle dit : merci. On ne rit pas des lunettes, des cheveux ou d'un habit. On ne va pas rire de l'apparence. On joue. La cloche de la récréation sonne. Dans la cour, Inès et Lila courent vers le cerceau. Lila met le cerceau à terre. Elles sautent dedans, une après l'autre. Les lunettes restent sur le nez de Lila. Les cheveux bougent. Le manteau bleu reste boutonné. Le jeu continue. Inès dit : encore. Lila dit : encore. [pause]</t>
+          <t>La laine des manteaux sent la pluie. Ça sent mouillé, maman. Tu le sens, sur le tissu ? Oui, un peu froid. Le radiateur fait un tic chaud. Tu l'entends, près des crochets ? Oui, papa. Papa égoutte un manteau, sans parler. Une botte jaune est couchée. Sur le caoutchouc, un &lt;emphasis&gt;éclat de botte&lt;/emphasis&gt; luit. Il brille, papa ! Tu le vois, sur la botte ? Oui, un petit point. Une goutte tombe du capuchon. Elle fait un rond sur le bois. Le bois est luisant. La pluie a fini, dehors. La cour brille. Il y a une flaque, Mila. Je veux un bateau, maintenant ! Un bateau de papier ? Oui, pour la flaque. Maman pose une feuille blanche. La feuille est un peu rêche. Elle sent le bois. Tu restes près des bottes ? Oui, papa. En ce moment, Mila plie la feuille trop vite. Un coin se replie tout seul. Il penche ! Le milieu, Mila ? J'y vais. Sarah arrive près des bottes. Son manteau est bleu vif. Sarah a les cheveux courts. Sarah ! Sarah a des lunettes. Elles brillent un peu. Elles brillent ! Mila avance la main vers les lunettes. Non. Sarah recule d'un pas. Oh. Mila plie toute seule, trop vite. Le papier fait frrt. Le bateau penche, de travers. Il ne tient pas. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'éclat de botte tremble, puis tient. Tu vois Sarah, Mila ? Papa s'accroupit à la même hauteur. Oui, papa. Tes mains sont froides, Mila ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>éclat de botte</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,54 +1321,73 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_bateau_et_sarah_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le radiateur de l'entrée fait un tic chaud.
-narrateur|Les manteaux sentent la laine mouillée.
+          <t>narrateur|La laine des manteaux sent la pluie.
+enfant-f|Ça sent mouillé, maman.
+maman|Tu le sens, sur le tissu ?
+enfant-f|Oui, un peu froid.
+narrateur|Le radiateur fait un tic chaud.
+papa|Tu l'entends, près des crochets ?
+enfant-f|Oui, papa.
+narrateur|Papa égoutte un manteau, sans parler.
 narrateur|Une botte jaune est couchée.
+narrateur|Sur le caoutchouc, un éclat de botte luit.
+enfant-f|Il brille, papa !
+papa|Tu le vois, sur la botte ?
+enfant-f|Oui, un petit point.
 narrateur|Une goutte tombe du capuchon.
 narrateur|Elle fait un rond sur le bois.
+enfant-f|Le bois est luisant.
+maman|La pluie a fini, dehors.
+enfant-f|La cour brille.
+papa|Il y a une flaque, Mila.
+enfant-f|Je veux un bateau, maintenant !
+maman|Un bateau de papier ?
+enfant-f|Oui, pour la flaque.
 narrateur|Maman pose une feuille blanche.
 narrateur|La feuille est un peu rêche.
-maman|Tu as entendu le radiateur, Mila ?
-enfant-f|Il fait tic.
-maman|Oui.
-maman|Il réchauffe les manteaux.
-narrateur|En ce moment, Mila plie la feuille.
-narrateur|Elle veut un bateau.
-enfant-f|Il va flotter.
-enfant-f|Dans la flaque.
-maman|On plie bien le milieu ?
-enfant-f|Oui.
-narrateur|Le papier sent le bois.
+enfant-f|Elle sent le bois.
+papa|Tu restes près des bottes ?
+enfant-f|Oui, papa.
+narrateur|En ce moment, Mila plie la feuille trop vite.
 narrateur|Un coin se replie tout seul.
-narrateur|Mila l'aplatit avec la main.
+enfant-f|Il penche !
+maman|Le milieu, Mila ?
+enfant-f|J'y vais.
 narrateur|Sarah arrive près des bottes.
-narrateur|Sarah a des lunettes neuves.
+narrateur|Son manteau est bleu vif.
+narrateur|Sarah a les cheveux courts.
+enfant-f|Sarah !
+narrateur|Sarah a des lunettes.
 narrateur|Elles brillent un peu.
-narrateur|Sarah a les cheveux courts.
-narrateur|Son manteau est bleu vif.
-maman|Venez plier toutes les deux.
-enfant-f|Tu m'aides, Sarah ?
-copine|Oui.
-narrateur|Elles plient encore.
+enfant-f|Elles brillent !
+narrateur|Mila avance la main vers les lunettes.
+copine|Non.
+narrateur|Sarah recule d'un pas.
+enfant-f|Oh.
+narrateur|Mila plie toute seule, trop vite.
 narrateur|Le papier fait frrt.
-narrateur|Un pli est trop haut.
-narrateur|L'autre pli est trop bas.
-narrateur|Le bateau est un peu de travers.
-enfant-f|Il penche.
-maman|On peut regarder le pli.
-narrateur|Sarah se penche.
-narrateur|Ses lunettes aident à voir.
-copine|Là.
-copine|Ce pli-là.
-enfant-f|Je le vois.</t>
+narrateur|Le bateau penche, de travers.
+enfant-f|Il ne tient pas.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|L'éclat de botte tremble, puis tient.
+papa|Tu vois Sarah, Mila ?
+narrateur|Papa s'accroupit à la même hauteur.
+enfant-f|Oui, papa.
+maman|Tes mains sont froides, Mila ?
+enfant-f|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>feuilles</t>
+          <t>feuilles,manteaux</t>
         </is>
       </c>
     </row>
@@ -1400,12 +1419,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah a des lunettes. Que fait Mila ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah a des &lt;emphasis level="moderate"&gt;lunettes&lt;/emphasis&gt;. Que fait Mila ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lila a des lunettes. Que fait-on ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah a des &lt;emphasis&gt;lunettes&lt;/emphasis&gt;. Que fait Mila ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1468,7 +1487,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1479,7 +1498,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1494,34 +1513,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>lunettes</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1536,17 +1559,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=mila_plie_avec_sarah_sans_commenter; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1579,17 +1602,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila écoute Sarah. Elles replient le milieu. Vous pliez ensemble. Merci, Mila. Merci, Sarah. Le bateau se tient droit. Il est prêt. On va à la flaque ? On met les bottes d'abord. Mila enfile la botte jaune. Sarah enfile les siennes. Le caoutchouc est un peu froid. Elle colle, maman. Tire doucement. Sarah a vu le pli. Le bateau se tient. J'ouvre la porte ? Oui. La poignée est froide. L'air de la cour entre.</t>
+          <t>Mila avance trop vite vers la feuille. Tu plies, maintenant ! Les mots se bousculent dans sa bouche. Non. Sarah reste près des bottes. Oh. Le sourire ne revient pas. Mila refuse de foncer. Elle referme la main. Tu veux le bateau avec Sarah ? Papa reste à la même hauteur. Tu regardes ? Sarah ne dit rien, d'abord. Elle pose un genou près du bois. Je plie. D'accord. Merci, Mila. Papa a vu les deux, près de la feuille. Le papier est rêche, sous les doigts. Il sent le bois. Elles replient le milieu, sans se presser. Sarah montre un pli, du doigt. Là. Je le vois. Le bateau se tient droit. Il est prêt ! La flaque ? Les bottes d'abord, Mila. Mila enfile la botte jaune. Sarah enfile les siennes. Elle colle, maman. Tire un peu. Elle vient. La poignée est froide, toi ? Oui, papa. J'ouvre ? Oui. L'air de la cour entre. Ça sent la pluie. La flaque est là. On y va. Le ventre de Mila se desserre. Les épaules se relèvent un peu.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila écoute Sarah. Elles replient le milieu. Vous pliez ensemble. Merci, Mila. Merci, Sarah. Le bateau se tient droit. Il est prêt. On va à la flaque ? On met les bottes d'abord. Mila enfile la botte jaune. Sarah enfile les siennes. Le caoutchouc est un peu froid. Elle colle, maman. Tire doucement. Sarah a vu le pli. Le bateau se tient. J'ouvre la porte ? Oui. La poignée est froide. L'air de la cour entre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila avance trop vite vers la feuille. Tu plies, maintenant ! Les mots se bousculent dans sa bouche. Non. Sarah reste près des bottes. Oh. Le sourire ne revient pas. Mila refuse de foncer. Elle referme la main. Tu veux le bateau avec Sarah ? Papa reste à la même hauteur. Tu regardes ? Sarah ne dit rien, d'abord. Elle pose un genou près du bois. Je plie. &lt;emphasis level="moderate"&gt;D'accord&lt;/emphasis&gt;. Merci, Mila. Papa a vu les deux, près de la feuille. Le papier est rêche, sous les doigts. Il sent le bois. Elles replient le milieu, sans se presser. Sarah montre un pli, du doigt. Là. Je le vois. Le bateau se tient droit. Il est prêt ! La flaque ? Les bottes d'abord, Mila. Mila enfile la botte jaune. Sarah enfile les siennes. Elle colle, maman. Tire un peu. Elle vient. La poignée est froide, toi ? Oui, papa. J'ouvre ? Oui. L'air de la cour entre. Ça sent la pluie. La flaque est là. On y va. Le ventre de Mila se desserre. Les épaules se relèvent un peu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Inès a entendu maman. On ne va &lt;emphasis&gt;pas&lt;/emphasis&gt; rire de l'apparence. Inès a invité Lila. Elles ont joué. [pause]</t>
+          <t>Mila avance trop vite vers la feuille. Tu plies, maintenant ! Les mots se bousculent dans sa bouche. Non. Sarah reste près des bottes. Oh. Le sourire ne revient pas. Mila refuse de foncer. Elle referme la main. Tu veux le bateau avec Sarah ? Papa reste à la même hauteur. Tu regardes ? Sarah ne dit rien, d'abord. Elle pose un genou près du bois. Je plie. &lt;emphasis&gt;D'accord&lt;/emphasis&gt;. Merci, Mila. Papa a vu les deux, près de la feuille. Le papier est rêche, sous les doigts. Il sent le bois. Elles replient le milieu, sans se presser. Sarah montre un pli, du doigt. Là. Je le vois. Le bateau se tient droit. Il est prêt ! La flaque ? Les bottes d'abord, Mila. Mila enfile la botte jaune. Sarah enfile les siennes. Elle colle, maman. Tire un peu. Elle vient. La poignée est froide, toi ? Oui, papa. J'ouvre ? Oui. L'air de la cour entre. Ça sent la pluie. La flaque est là. On y va. Le ventre de Mila se desserre. Les épaules se relèvent un peu. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1636,7 +1659,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1644,10 +1667,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1670,30 +1693,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>D'accord</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1702,10 +1725,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1718,31 +1741,59 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_le_silence_puis_dit_d_accord; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila écoute Sarah.
-narrateur|Elles replient le milieu.
-maman|Vous pliez ensemble.
-maman|Merci, Mila.
-maman|Merci, Sarah.
+          <t>narrateur|Mila avance trop vite vers la feuille.
+enfant-f|Tu plies, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+copine|Non.
+narrateur|Sarah reste près des bottes.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Mila refuse de foncer.
+narrateur|Elle referme la main.
+papa|Tu veux le bateau avec Sarah ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Tu regardes ?
+narrateur|Sarah ne dit rien, d'abord.
+narrateur|Elle pose un genou près du bois.
+copine|Je plie.
+enfant-f|D'accord.
+papa|Merci, Mila.
+narrateur|Papa a vu les deux, près de la feuille.
+maman|Le papier est rêche, sous les doigts.
+enfant-f|Il sent le bois.
+narrateur|Elles replient le milieu, sans se presser.
+narrateur|Sarah montre un pli, du doigt.
+copine|Là.
+enfant-f|Je le vois.
 narrateur|Le bateau se tient droit.
-enfant-f|Il est prêt.
-copine|On va à la flaque ?
-maman|On met les bottes d'abord.
+enfant-f|Il est prêt !
+copine|La flaque ?
+maman|Les bottes d'abord, Mila.
 narrateur|Mila enfile la botte jaune.
 narrateur|Sarah enfile les siennes.
-narrateur|Le caoutchouc est un peu froid.
 enfant-f|Elle colle, maman.
-maman|Tire doucement.
-maman|Sarah a vu le pli.
-maman|Le bateau se tient.
-enfant-f|J'ouvre la porte ?
+maman|Tire un peu.
+enfant-f|Elle vient.
+papa|La poignée est froide, toi ?
+enfant-f|Oui, papa.
+enfant-f|J'ouvre ?
 maman|Oui.
-narrateur|La poignée est froide.
-narrateur|L'air de la cour entre.</t>
+narrateur|L'air de la cour entre.
+enfant-f|Ça sent la pluie.
+papa|La flaque est là.
+enfant-f|On y va.
+narrateur|Le ventre de Mila se desserre.
+narrateur|Les épaules se relèvent un peu.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>papier</t>
         </is>
       </c>
     </row>
@@ -1769,17 +1820,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>La cour brille encore. La flaque est ronde et calme. Mila pose le bateau. Le papier tremble. Il flotte ! Il avance. Bravo. Vous avez bien plié. Elles soufflent tout doux. La voile se gonfle un peu. Le bateau tourne dans l'eau. Encore un souffle. Le mien aussi. Sarah souffle à son tour. Une petite vague arrive. Il reste droit. Grâce au pli. Oui. Sarah l'a vu. Une feuille sèche passe sur l'eau. Le bateau l'évite. Il est fort. C'est notre bateau. Le radiateur tic encore, derrière.</t>
+          <t>La cour brille, après la pluie. La flaque est ronde, un peu lisse. Je le mets, d'un coup ! Mila pose le bateau trop vite. Le papier tremble, puis s'arrête au bord. Il n'avance pas ! Attends. Sarah reste un pas plus loin. Mila avance la main, trop vite. Tu souffles, maintenant ! Non. Oh. Le bateau reste collé au bord. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle observe la flaque, un instant. J'écoute. Elle écoute le tic, derrière la porte. Sur le caoutchouc, un éclat de botte luit. Là, sur la botte. Tu souffles, si tu veux ? Sarah ne dit rien. Elle se baisse près de l'eau. Oui. Elles soufflent, sans se presser. La voile se gonfle un peu. Il avance ! Il tourne. Tu le vois, au milieu ? Oui, papa. Une feuille passe sur l'eau. Il l'évite. Il est fort. C'est notre bateau. Tu restes un peu ? Oui, papa. Tes bottes sont froides ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>La cour brille encore. La flaque est ronde et calme. Mila pose le bateau. Le papier tremble. Il flotte ! Il avance. Bravo. Vous avez bien plié. Elles soufflent tout doux. La voile se gonfle un peu. Le bateau tourne dans l'eau. Encore un souffle. Le mien aussi. Sarah souffle à son tour. Une petite vague arrive. Il reste droit. Grâce au pli. Oui. Sarah l'a vu. Une feuille sèche passe sur l'eau. Le bateau l'évite. Il est fort. C'est notre bateau. Le radiateur tic encore, derrière.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La cour brille, après la pluie. La flaque est ronde, un peu lisse. Je le mets, d'un coup ! Mila pose le bateau trop vite. Le papier tremble, puis s'arrête au bord. Il n'avance pas ! Attends. Sarah reste un pas plus loin. Mila avance la main, trop vite. Tu souffles, maintenant ! Non. Oh. Le bateau reste collé au bord. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle observe la flaque, un instant. J'écoute. Elle écoute le tic, derrière la porte. Sur le caoutchouc, un &lt;emphasis level="moderate"&gt;éclat de botte&lt;/emphasis&gt; luit. Là, sur la botte. Tu souffles, si tu veux ? Sarah ne dit rien. Elle se baisse près de l'eau. Oui. Elles soufflent, sans se presser. La voile se gonfle un peu. Il avance ! Il tourne. Tu le vois, au milieu ? Oui, papa. Une feuille passe sur l'eau. Il l'évite. Il est fort. C'est notre bateau. Tu restes un peu ? Oui, papa. Tes bottes sont froides ? Un peu, maman.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>La cloche sonne la fin. Maman revient près du portail. Inès et Lila se disent à de&lt;emphasis&gt;main&lt;/emphasis&gt;. Le manteau bleu part dans la rue. [pause]</t>
+          <t>&lt;low-pitch&gt;La cour brille, après la pluie. La flaque est ronde, un peu lisse. Je le mets, d'un coup ! Mila pose le bateau trop vite. Le papier tremble, puis s'arrête au bord. Il n'avance pas ! Attends. Sarah reste un pas plus loin. Mila avance la main, trop vite. Tu souffles, maintenant ! Non. Oh. Le bateau reste collé au bord. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle observe la flaque, un instant. J'écoute. Elle écoute le tic, derrière la porte. Sur le caoutchouc, un &lt;emphasis&gt;éclat de botte&lt;/emphasis&gt; luit. Là, sur la botte. Tu souffles, si tu veux ? Sarah ne dit rien. Elle se baisse près de l'eau. Oui. Elles soufflent, sans se presser. La voile se gonfle un peu. Il avance ! Il tourne. Tu le vois, au milieu ? Oui, papa. Une feuille passe sur l'eau. Il l'évite. Il est fort. C'est notre bateau. Tu restes un peu ? Oui, papa. Tes bottes sont froides ? Un peu, maman.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1826,7 +1877,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1834,22 +1885,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1860,30 +1915,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de botte</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1892,47 +1947,70 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat_de_botte; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|La cour brille encore.
-narrateur|La flaque est ronde et calme.
-narrateur|Mila pose le bateau.
-narrateur|Le papier tremble.
-enfant-f|Il flotte !
-copine|Il avance.
-maman|Bravo.
-maman|Vous avez bien plié.
-narrateur|Elles soufflent tout doux.
+          <t>narrateur|La cour brille, après la pluie.
+narrateur|La flaque est ronde, un peu lisse.
+enfant-f|Je le mets, d'un coup !
+narrateur|Mila pose le bateau trop vite.
+narrateur|Le papier tremble, puis s'arrête au bord.
+enfant-f|Il n'avance pas !
+copine|Attends.
+narrateur|Sarah reste un pas plus loin.
+narrateur|Mila avance la main, trop vite.
+enfant-f|Tu souffles, maintenant !
+copine|Non.
+enfant-f|Oh.
+narrateur|Le bateau reste collé au bord.
+narrateur|Mila refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Elle observe la flaque, un instant.
+enfant-f|J'écoute.
+narrateur|Elle écoute le tic, derrière la porte.
+narrateur|Sur le caoutchouc, un éclat de botte luit.
+enfant-f|Là, sur la botte.
+enfant-f|Tu souffles, si tu veux ?
+narrateur|Sarah ne dit rien.
+narrateur|Elle se baisse près de l'eau.
+copine|Oui.
+narrateur|Elles soufflent, sans se presser.
 narrateur|La voile se gonfle un peu.
-narrateur|Le bateau tourne dans l'eau.
-enfant-f|Encore un souffle.
-copine|Le mien aussi.
-narrateur|Sarah souffle à son tour.
-narrateur|Une petite vague arrive.
-maman|Il reste droit.
-enfant-f|Grâce au pli.
-maman|Oui.
-maman|Sarah l'a vu.
-narrateur|Une feuille sèche passe sur l'eau.
-narrateur|Le bateau l'évite.
+enfant-f|Il avance !
+copine|Il tourne.
+papa|Tu le vois, au milieu ?
+enfant-f|Oui, papa.
+maman|Une feuille passe sur l'eau.
+enfant-f|Il l'évite.
 copine|Il est fort.
 enfant-f|C'est notre bateau.
-narrateur|Le radiateur tic encore, derrière.</t>
+papa|Tu restes un peu ?
+enfant-f|Oui, papa.
+maman|Tes bottes sont froides ?
+enfant-f|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>eau,papier</t>
         </is>
       </c>
     </row>
@@ -1959,17 +2037,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau tourne au milieu. La botte jaune attend près du seuil. Il a flotté. Oui. Vous avez plié le bateau. La laine sèche tout doux.</t>
+          <t>Le bateau a flotté, papa. Tu le vois, comme tout à l'heure ? Oui, au milieu. On le garde près de nous ? Oui, maman. La botte jaune attend près du seuil. Elle est tiède. Le caoutchouc luit, toi ? Un peu, papa. Mila pose un doigt sur la botte. Ça sentait la laine. Les manteaux sèchent, près du radiateur. Il fait tic. On reste un peu ? Oui. Les joues de Mila se réchauffent. Il tourne. Oui. Le papier reste mouillé, au milieu. Un éclat de botte reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau tourne au milieu. La botte jaune attend près du seuil. Il a flotté. Oui. Vous avez plié le bateau. La laine sèche tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le bateau a flotté, papa. Tu le vois, comme tout à l'heure ? Oui, au milieu. On le garde près de nous ? Oui, maman. La botte jaune attend près du seuil. Elle est tiède. Le caoutchouc luit, toi ? Un peu, papa. Mila pose un doigt sur la botte. Ça sentait la laine. Les manteaux sèchent, près du radiateur. Il fait tic. On reste un peu ? Oui. Les joues de Mila se réchauffent. Il tourne. Oui. Le papier reste mouillé, au milieu. Un &lt;emphasis level="moderate"&gt;éclat de botte&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le bateau a flotté, papa. Tu le vois, comme tout à l'heure ? Oui, au milieu. On le garde près de nous ? Oui, maman. La botte jaune attend près du seuil. Elle est tiède. Le caoutchouc luit, toi ? Un peu, papa. Mila pose un doigt sur la botte. Ça sentait la laine. Les manteaux sèchent, près du radiateur. Il fait tic. On reste un peu ? Oui. Les joues de Mila se réchauffent. Il tourne. Oui. Le papier reste mouillé, au milieu. Un &lt;emphasis&gt;éclat de botte&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2016,18 +2094,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2036,12 +2114,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2050,17 +2128,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de botte</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2069,11 +2151,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2082,29 +2164,52 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_botte_reste_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le bateau tourne au milieu.
+          <t>enfant-f|Le bateau a flotté, papa.
+papa|Tu le vois, comme tout à l'heure ?
+enfant-f|Oui, au milieu.
+maman|On le garde près de nous ?
+enfant-f|Oui, maman.
 narrateur|La botte jaune attend près du seuil.
-enfant-f|Il a flotté.
-maman|Oui.
-maman|Vous avez plié le bateau.
-narrateur|La laine sèche tout doux.</t>
+enfant-f|Elle est tiède.
+papa|Le caoutchouc luit, toi ?
+enfant-f|Un peu, papa.
+narrateur|Mila pose un doigt sur la botte.
+enfant-f|Ça sentait la laine.
+maman|Les manteaux sèchent, près du radiateur.
+enfant-f|Il fait tic.
+papa|On reste un peu ?
+enfant-f|Oui.
+narrateur|Les joues de Mila se réchauffent.
+copine|Il tourne.
+enfant-f|Oui.
+narrateur|Le papier reste mouillé, au milieu.
+narrateur|Un éclat de botte reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>radiateur</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2210,6 +2315,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>